<commit_message>
Update hero slide titles to exact concise titles requested
</commit_message>
<xml_diff>
--- a/Hero Slides Updated.xlsx
+++ b/Hero Slides Updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\surya\OneDrive\ONE DRIVE\Desktop\LorVen Wesbsite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DB58970-6110-4854-B2AF-A03131ABA671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A4DC12D-32C4-4D95-9188-BD65AAFA3309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,36 +52,21 @@
     <t>Training Simulators</t>
   </si>
   <si>
-    <t>WLI — IoT-Based Water Level Indicator</t>
-  </si>
-  <si>
     <t>Real-time water-tank level measurement for passenger coaches, reported coach-wise to the CRIS server — enabling planned watering at nominated stations and reducing en-route watering failures.</t>
   </si>
   <si>
-    <t>IFD — Intelligent Field Device for IR-NIYANTRAC</t>
-  </si>
-  <si>
     <t>Real-time monitoring, energy metering and remote control of railway electrical assets — reporting to IR-NIYANTRAC over the oneM2M Common Service Platform as per IS/RDSO-PSE/1004:2026 (Rev-0).</t>
   </si>
   <si>
-    <t>RDPMS — Remote Diagnostic &amp; Predictive Maintenance</t>
-  </si>
-  <si>
     <t>IoT-based condition monitoring and predictive maintenance for Indian Railways signalling assets — diagnostic logic and AI/ML analytics generate maintenance alerts before failures occur (RDSO/SPN/257/2025).</t>
   </si>
   <si>
-    <t>IPS — SMPS-Based Integrated Power Supply</t>
-  </si>
-  <si>
     <t>Continuous, regulated AC and DC power for railway signalling circuits in RE and Non-RE areas — Stations, LC Gates, IBH and Auto Huts as per RDSO Specification RDSO/SPN/165/2023, Version 4.0.</t>
   </si>
   <si>
     <t>For every train passing a monitoring point, AHABD establishes which coach each temperature reading belongs to — delivering a complete, identified record of the pass and flagging overheating for attention.</t>
   </si>
   <si>
-    <t>Driving Simulators for Loco Pilots</t>
-  </si>
-  <si>
     <t>For Loco Pilots and Assistant Loco Pilots — three-phase electric locomotives (WAP/WAG) and train sets: EMU, MEMU and Vande Bharat. Developed in line with RDSO functional requirements.</t>
   </si>
   <si>
@@ -148,7 +133,22 @@
     <t>Advanced simulation platforms for Driving Simulators and KAVACH Training Simulators, delivering realistic operator training, enhanced safety, and operational readiness.</t>
   </si>
   <si>
-    <t>AHABD — Advancned Hot Axle Box Detection</t>
+    <t>Water Level Indicator</t>
+  </si>
+  <si>
+    <t>Intelligent Field Device for IR-NIYANTRAC</t>
+  </si>
+  <si>
+    <t>RDPMS</t>
+  </si>
+  <si>
+    <t>IPS</t>
+  </si>
+  <si>
+    <t>Advancned Hot Axle Box Detection</t>
+  </si>
+  <si>
+    <t>Driving Simulators</t>
   </si>
 </sst>
 </file>
@@ -563,7 +563,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -574,7 +574,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -596,7 +596,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -607,7 +607,7 @@
         <v>8</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -615,10 +615,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -629,7 +629,7 @@
         <v>9</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -637,10 +637,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -648,10 +648,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -659,10 +659,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -670,10 +670,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -681,10 +681,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -692,10 +692,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -703,10 +703,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -714,10 +714,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -725,10 +725,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -736,10 +736,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -747,10 +747,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -758,10 +758,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -769,10 +769,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>